<commit_message>
Mise à jour du Gantt
J'ai terminé mon planning.
</commit_message>
<xml_diff>
--- a/Gantt.xlsx
+++ b/Gantt.xlsx
@@ -1,47 +1,64 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\BUT3\S5\Visualisation\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Utilisateur\Desktop\Chaïma\Site PORTFOLIO\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{661ED4B4-CE6E-4399-B8C2-471E9D0D458D}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA2EF8B2-CA31-4434-AFDF-D2B218ED7DDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19095" yWindow="0" windowWidth="19410" windowHeight="20985" xr2:uid="{7CDCFAC3-7FE8-4EFA-B0B6-49296FA54FD1}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{7CDCFAC3-7FE8-4EFA-B0B6-49296FA54FD1}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="25">
   <si>
     <t>TÂCHE</t>
   </si>
   <si>
+    <t>DATE DÉBUT</t>
+  </si>
+  <si>
+    <t>DATE FIN</t>
+  </si>
+  <si>
     <t>AVANCEMENT</t>
   </si>
   <si>
+    <t>INITIALISATION</t>
+  </si>
+  <si>
+    <t>Création du projet GIT</t>
+  </si>
+  <si>
     <t>Terminée</t>
   </si>
   <si>
-    <t>Création du projet GIT</t>
-  </si>
-  <si>
     <t>Dépôt du lien</t>
   </si>
   <si>
@@ -51,47 +68,56 @@
     <t>Réalisation de la maquette</t>
   </si>
   <si>
-    <t>En cours</t>
-  </si>
-  <si>
-    <t>Débutée</t>
-  </si>
-  <si>
-    <t>DATE DÉBUT</t>
-  </si>
-  <si>
-    <t>INITIALISATION</t>
+    <t>CONCEPTION</t>
   </si>
   <si>
     <t>Développement partie serveur</t>
   </si>
   <si>
+    <t>Visualisations</t>
+  </si>
+  <si>
     <t>Intégration des parties</t>
   </si>
   <si>
-    <t>CONCEPTION</t>
-  </si>
-  <si>
-    <t>DATE FIN</t>
-  </si>
-  <si>
-    <t>Visualisations</t>
-  </si>
-  <si>
     <t>AMÉLIORATIONS</t>
   </si>
   <si>
-    <t>Amélioration du site</t>
-  </si>
-  <si>
-    <t>Amélioration du planning</t>
+    <t>Rédaction ReadMe principal</t>
+  </si>
+  <si>
+    <t>Choix et préparation des données</t>
+  </si>
+  <si>
+    <t>Architecture du site</t>
+  </si>
+  <si>
+    <t>Créaion pages HTML et menu</t>
+  </si>
+  <si>
+    <t>Mise en forme (CSS)</t>
+  </si>
+  <si>
+    <t>Ajout des interactions</t>
+  </si>
+  <si>
+    <t>Tests et corrections</t>
+  </si>
+  <si>
+    <t>Amélioration du site (design, version mobile)</t>
+  </si>
+  <si>
+    <t>Mise à jour du planning</t>
+  </si>
+  <si>
+    <t>Pas encore débutée</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -182,17 +208,14 @@
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="3" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
@@ -202,10 +225,22 @@
     <xf numFmtId="14" fontId="1" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFill="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="3" applyFont="1" applyFill="1">
-      <alignment horizontal="left" vertical="center" indent="2"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="3" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyFill="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
   </cellXfs>
@@ -545,142 +580,278 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F8D3A4A-0E23-490F-8C22-A2EAAA8FF501}">
-  <dimension ref="A1:D13"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.25"/>
+  <dimension ref="A1:D20"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="3" width="28.625" customWidth="1"/>
+    <col min="1" max="1" width="28.5703125" style="10" customWidth="1"/>
+    <col min="2" max="3" width="28.5703125" customWidth="1"/>
     <col min="4" max="4" width="27" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" thickBot="1">
-      <c r="A1" s="4" t="s">
+    <row r="1" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D1" s="5" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A2" s="1" t="s">
-        <v>10</v>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="7" t="s">
+        <v>4</v>
       </c>
       <c r="B2" s="1"/>
       <c r="C2" s="1"/>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" ht="15" thickBot="1">
-      <c r="A3" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="B3" s="6">
+    <row r="3" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="8" t="s">
+        <v>5</v>
+      </c>
+      <c r="B3" s="5">
         <v>46301</v>
       </c>
-      <c r="C3" s="6">
+      <c r="C3" s="5">
         <v>46301</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15" thickBot="1">
-      <c r="A4" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B4" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="5">
         <v>46301</v>
       </c>
-      <c r="C4" s="6">
+      <c r="C4" s="5">
         <v>46301</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15" thickBot="1">
-      <c r="A5" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="B5" s="6">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="B5" s="5">
         <v>46301</v>
       </c>
-      <c r="C5" s="6"/>
+      <c r="C5" s="5">
+        <v>46304</v>
+      </c>
       <c r="D5" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15" thickBot="1">
-      <c r="A6" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="6">
+    </row>
+    <row r="6" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="5">
         <v>46301</v>
       </c>
-      <c r="C6" s="6"/>
+      <c r="C6" s="5">
+        <v>46301</v>
+      </c>
       <c r="D6" s="2" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A7" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46304</v>
+      </c>
+      <c r="C7" s="5">
+        <v>46304</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B8" s="1"/>
+      <c r="C8" s="1"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9" s="11">
+        <v>46307</v>
+      </c>
+      <c r="C9" s="11">
+        <v>46317</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="B10" s="11">
+        <v>46318</v>
+      </c>
+      <c r="C10" s="11">
+        <v>46332</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="B11" s="11">
+        <v>46321</v>
+      </c>
+      <c r="C11" s="11">
+        <v>46339</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="11">
+        <v>46335</v>
+      </c>
+      <c r="C12" s="11">
+        <v>46346</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>11</v>
+      </c>
+      <c r="B13" s="11">
+        <v>46349</v>
+      </c>
+      <c r="C13" s="11">
+        <v>46356</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46350</v>
+      </c>
+      <c r="C14" s="5">
+        <v>46360</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46356</v>
+      </c>
+      <c r="C15" s="5">
+        <v>46365</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="2"/>
-    </row>
-    <row r="8" spans="1:4" ht="15" thickBot="1">
-      <c r="A8" s="7" t="s">
-        <v>11</v>
-      </c>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="2"/>
-    </row>
-    <row r="9" spans="1:4" ht="15" thickBot="1">
-      <c r="A9" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="B9" s="3"/>
-      <c r="C9" s="3"/>
-      <c r="D9" s="2"/>
-    </row>
-    <row r="10" spans="1:4" ht="15" thickBot="1">
-      <c r="A10" s="7" t="s">
-        <v>12</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="2"/>
-    </row>
-    <row r="11" spans="1:4" ht="15.75" thickBot="1">
-      <c r="A11" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="2"/>
-    </row>
-    <row r="12" spans="1:4" ht="15" thickBot="1">
-      <c r="A12" s="7" t="s">
-        <v>17</v>
-      </c>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="2"/>
-    </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="8" t="s">
-        <v>18</v>
+      <c r="B16" s="5">
+        <v>46356</v>
+      </c>
+      <c r="C16" s="5">
+        <v>46367</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" s="1"/>
+      <c r="C17" s="1"/>
+      <c r="D17" s="2"/>
+    </row>
+    <row r="18" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="9" t="s">
+        <v>21</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46363</v>
+      </c>
+      <c r="C18" s="5">
+        <v>46374</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46391</v>
+      </c>
+      <c r="C19" s="5">
+        <v>46409</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B20" s="5">
+        <v>46666</v>
+      </c>
+      <c r="C20" s="5">
+        <v>46409</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>24</v>
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="D2:D12">
+  <conditionalFormatting sqref="D2:D20">
     <cfRule type="dataBar" priority="1">
       <dataBar>
         <cfvo type="num" val="0"/>
@@ -695,7 +866,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D3:D6 D8:D10 D12" xr:uid="{D95B77AE-E663-4420-A926-D29DD3373C3D}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="D9:D16 D3:D7 D18:D20" xr:uid="{D95B77AE-E663-4420-A926-D29DD3373C3D}">
       <formula1>"Pas encore débutée,Débutée,En cours,Finalisation,Terminée"</formula1>
     </dataValidation>
   </dataValidations>
@@ -716,7 +887,7 @@
               <x14:axisColor rgb="FF000000"/>
             </x14:dataBar>
           </x14:cfRule>
-          <xm:sqref>D2:D12</xm:sqref>
+          <xm:sqref>D2:D20</xm:sqref>
         </x14:conditionalFormatting>
       </x14:conditionalFormattings>
     </ext>

</xml_diff>